<commit_message>
Update list and result Excel files with new data
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Randomizer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\projects\github.com\Demparty\an.mn\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DA764D-6DE5-40DB-B3D3-050B98070A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="list" sheetId="1" r:id="rId1"/>
@@ -19,38 +20,51 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>total_pool</t>
   </si>
   <si>
     <t>choose_pool</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>uuriin_hayg</t>
+  </si>
+  <si>
+    <t>test 1</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>test 3</t>
+  </si>
+  <si>
+    <t>test 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -411,51 +425,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="10.9375" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
         <v>15</v>
       </c>
-      <c r="B2">
+      <c r="D2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
         <v>20</v>
       </c>
-      <c r="B3">
+      <c r="D3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
         <v>13</v>
       </c>
-      <c r="B4">
+      <c r="D4">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
         <v>35</v>
       </c>
-      <c r="B5">
+      <c r="D5">
         <v>8</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance main.py to include block height and update column names; add new Excel files for list and result data.
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\projects\github.com\Demparty\an.mn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DA764D-6DE5-40DB-B3D3-050B98070A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9561DDAB-9C28-4AD9-8BA1-FC17D7639418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,22 +33,22 @@
     <t>choose_pool</t>
   </si>
   <si>
+    <t>uuriin_hayg</t>
+  </si>
+  <si>
+    <t>test 1</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>test 3</t>
+  </si>
+  <si>
+    <t>test 4</t>
+  </si>
+  <si>
     <t>id</t>
-  </si>
-  <si>
-    <t>uuriin_hayg</t>
-  </si>
-  <si>
-    <t>test 1</t>
-  </si>
-  <si>
-    <t>test 2</t>
-  </si>
-  <si>
-    <t>test 3</t>
-  </si>
-  <si>
-    <t>test 4</t>
   </si>
 </sst>
 </file>
@@ -431,10 +431,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>15</v>
@@ -462,7 +462,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -476,7 +476,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>13</v>
@@ -490,7 +490,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>35</v>

</xml_diff>

<commit_message>
Update .gitignore to retain result.xlsx and remove exclusion for *list.xlsx; update list.xlsx file
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\projects\github.com\Demparty\an.mn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9561DDAB-9C28-4AD9-8BA1-FC17D7639418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1593CB-B372-4199-9607-87A36F63F68A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,9 +33,6 @@
     <t>choose_pool</t>
   </si>
   <si>
-    <t>uuriin_hayg</t>
-  </si>
-  <si>
     <t>test 1</t>
   </si>
   <si>
@@ -49,6 +46,9 @@
   </si>
   <si>
     <t>id</t>
+  </si>
+  <si>
+    <t>sector_name</t>
   </si>
 </sst>
 </file>
@@ -431,10 +431,10 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
         <v>7</v>
-      </c>
-      <c r="B1" t="s">
-        <v>2</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>15</v>
@@ -462,7 +462,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>20</v>
@@ -476,7 +476,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4">
         <v>13</v>
@@ -490,7 +490,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>35</v>

</xml_diff>

<commit_message>
Add new Excel files (list1.xlsx, list2.xlsx, list3.xlsx, list4.xlsx) and update existing list.xlsx
</commit_message>
<xml_diff>
--- a/list.xlsx
+++ b/list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\projects\github.com\Demparty\an.mn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1593CB-B372-4199-9607-87A36F63F68A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5ACE5BE-C170-4492-B05E-AE54F0FB70E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>total_pool</t>
-  </si>
-  <si>
-    <t>choose_pool</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>test 1</t>
   </si>
@@ -49,6 +43,24 @@
   </si>
   <si>
     <t>sector_name</t>
+  </si>
+  <si>
+    <t>file_name</t>
+  </si>
+  <si>
+    <t>list1.xlsx</t>
+  </si>
+  <si>
+    <t>list2.xlsx</t>
+  </si>
+  <si>
+    <t>list3.xlsx</t>
+  </si>
+  <si>
+    <t>list4.xlsx</t>
+  </si>
+  <si>
+    <t>choose_count</t>
   </si>
 </sst>
 </file>
@@ -428,19 +440,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="10.9375" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="4.6875" customWidth="1"/>
+    <col min="2" max="2" width="12.9375" customWidth="1"/>
+    <col min="4" max="4" width="12.875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
       <c r="C1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.5">
@@ -448,13 +465,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>15</v>
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.5">
@@ -462,13 +479,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.5">
@@ -476,13 +493,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.5">
@@ -490,13 +507,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>35</v>
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>